<commit_message>
Enhance QR code lineage handling and tracking path functionality
- Updated the `TraceController` and `LotController` to utilize the new `QrCode::treeForApplication` method for improved lineage representation.
- Introduced a `trackingPaths` method in the `QrCode` model to generate paths for tracking roles, enhancing the clarity of QR code lineage.
- Modified the `lot-timeline` view to display tracking paths dynamically based on the nodes provided, improving user experience.
- Updated tests to verify the correct display of lineage and tracking paths in various scenarios.

These changes improve the visibility and usability of QR code lineage and tracking information in the application.
</commit_message>
<xml_diff>
--- a/docs/templates/import-akaun-penternak-pembekal.xlsx
+++ b/docs/templates/import-akaun-penternak-pembekal.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Senarai" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="Peranan">Senarai!$A$2:$A$3</definedName>
+    <definedName name="JenisRantaian">Senarai!$A$2:$A$5</definedName>
     <definedName name="Negeri">Senarai!$B$2:$B$17</definedName>
     <definedName name="PilihNegeri">Senarai!$S$2</definedName>
     <definedName name="Johor">Senarai!$C$2:$C$11</definedName>
@@ -89,23 +89,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1" style="2"/>
     <col min="3" max="3" width="36" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="34" customWidth="1"/>
-    <col min="8" max="8" width="42" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="10" width="28" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1" style="2"/>
-    <col min="12" max="12" width="16" customWidth="1" style="2"/>
-    <col min="13" max="13" width="32" customWidth="1"/>
-    <col min="14" max="14" width="28" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="34" customWidth="1"/>
+    <col min="9" max="9" width="42" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1" style="2"/>
+    <col min="13" max="13" width="16" customWidth="1" style="2"/>
+    <col min="14" max="14" width="32" customWidth="1"/>
+    <col min="15" max="15" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -131,66 +132,71 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peranan *</t>
+          <t xml:space="preserve">Jenis dalam rantaian *</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Nama lapisan</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">No. Pendaftaran *</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Nama Syarikat / Ladang *</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Alamat *</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Negeri</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Daerah</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Poskod</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">No. Telefon</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Emel Syarikat</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Laman Web</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
+  <autoFilter ref="A1:O1"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Peranan" prompt="Pilih Pembekal atau Penternak." errorTitle="Peranan" error="Pilih Pembekal atau Penternak dari senarai." sqref="E2:E500">
-      <formula1>Peranan</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Jenis dalam rantaian" prompt="Pilih Pengeluar, Pemborong, Peruncit, atau Lain-lain. Consumer tidak diisi di sini." errorTitle="Jenis dalam rantaian" error="Pilih jenis dari senarai." sqref="E2:E500">
+      <formula1>JenisRantaian</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Negeri" prompt="Pilih negeri atau wilayah persekutuan." errorTitle="Negeri" error="Pilih negeri dari senarai." sqref="I2:I500">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Negeri" prompt="Pilih negeri atau wilayah persekutuan." errorTitle="Negeri" error="Pilih negeri dari senarai." sqref="J2:J500">
       <formula1>Negeri</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Daerah" prompt="Pilih negeri pada baris ini dahulu. Senarai daerah mengikut negeri itu." errorTitle="Daerah" error="Pilih daerah dari senarai negeri ini." sqref="J2:J500">
-      <formula1>IF(I2="",PilihNegeri,INDIRECT(SUBSTITUTE(I2," ","_")))</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Daerah" prompt="Pilih negeri pada baris ini dahulu. Senarai daerah mengikut negeri itu." errorTitle="Daerah" error="Pilih daerah dari senarai negeri ini." sqref="K2:K500">
+      <formula1>IF(J2="",PilihNegeri,INDIRECT(SUBSTITUTE(J2," ","_")))</formula1>
     </dataValidation>
   </dataValidations>
 </worksheet>
@@ -198,23 +204,24 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1" style="2"/>
     <col min="3" max="3" width="36" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="34" customWidth="1"/>
-    <col min="8" max="8" width="42" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="10" width="28" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1" style="2"/>
-    <col min="12" max="12" width="16" customWidth="1" style="2"/>
-    <col min="13" max="13" width="32" customWidth="1"/>
-    <col min="14" max="14" width="28" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="34" customWidth="1"/>
+    <col min="9" max="9" width="42" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1" style="2"/>
+    <col min="13" max="13" width="16" customWidth="1" style="2"/>
+    <col min="14" max="14" width="32" customWidth="1"/>
+    <col min="15" max="15" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -240,50 +247,55 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peranan *</t>
+          <t xml:space="preserve">Jenis dalam rantaian *</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Nama lapisan</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">No. Pendaftaran *</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Nama Syarikat / Ladang *</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Alamat *</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Negeri</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Daerah</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Poskod</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">No. Telefon</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Emel Syarikat</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Laman Web</t>
         </is>
@@ -302,7 +314,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ahmad.penternak@example.com</t>
+          <t xml:space="preserve">ahmad.ladang@example.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -312,61 +324,62 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Penternak</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+          <t xml:space="preserve">Pengeluar</t>
+        </is>
+      </c>
+      <c r="F2"/>
+      <c r="G2" t="inlineStr">
         <is>
           <t xml:space="preserve">PTN-0001</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ladang Lembu Ahmad</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t xml:space="preserve">Lot 12, Jalan Ladang, Pontian</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t xml:space="preserve">Johor</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t xml:space="preserve">Pontian</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">82000</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">012-3456789</t>
         </is>
       </c>
-      <c r="M2"/>
       <c r="N2"/>
+      <c r="O2"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Siti binti Omar</t>
+          <t xml:space="preserve">Nora binti Karim</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">850202026666</t>
+          <t xml:space="preserve">810202026666</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">siti.pembekal@example.com</t>
+          <t xml:space="preserve">nora.borong@example.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -376,61 +389,127 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pembekal</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PMB-0001</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Pemborong</t>
+        </is>
+      </c>
+      <c r="F3"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pembekal Buah Siti</t>
+          <t xml:space="preserve">PBR-0001</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8, Jalan Pasar, Klang</t>
+          <t xml:space="preserve">Borong Buah Nora</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t xml:space="preserve">20, Jalan Gudang, Klang</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Selangor</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t xml:space="preserve">Klang</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">41000</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">019-1112223</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">siti@example.com</t>
-        </is>
-      </c>
-      <c r="N3"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nora@example.com</t>
+        </is>
+      </c>
+      <c r="O3"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aina binti Rahim</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">820303037777</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">aina.runcit@example.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tukar123!</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peruncit</t>
+        </is>
+      </c>
+      <c r="F4"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RNC-0001</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Runcit Segar Aina</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8, Jalan Pasar, Melaka</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Melaka</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Melaka Tengah</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">75000</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">012-8887766</t>
+        </is>
+      </c>
+      <c r="N4"/>
+      <c r="O4"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Peranan" prompt="Pilih Pembekal atau Penternak." errorTitle="Peranan" error="Pilih Pembekal atau Penternak dari senarai." sqref="E2:E20">
-      <formula1>Peranan</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Jenis dalam rantaian" prompt="Pilih Pengeluar, Pemborong, Peruncit, atau Lain-lain. Consumer tidak diisi di sini." errorTitle="Jenis dalam rantaian" error="Pilih jenis dari senarai." sqref="E2:E20">
+      <formula1>JenisRantaian</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Negeri" prompt="Pilih negeri atau wilayah persekutuan." errorTitle="Negeri" error="Pilih negeri dari senarai." sqref="I2:I20">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Negeri" prompt="Pilih negeri atau wilayah persekutuan." errorTitle="Negeri" error="Pilih negeri dari senarai." sqref="J2:J20">
       <formula1>Negeri</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Daerah" prompt="Pilih negeri pada baris ini dahulu. Senarai daerah mengikut negeri itu." errorTitle="Daerah" error="Pilih daerah dari senarai negeri ini." sqref="J2:J20">
-      <formula1>IF(I2="",PilihNegeri,INDIRECT(SUBSTITUTE(I2," ","_")))</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Daerah" prompt="Pilih negeri pada baris ini dahulu. Senarai daerah mengikut negeri itu." errorTitle="Daerah" error="Pilih daerah dari senarai negeri ini." sqref="K2:K20">
+      <formula1>IF(J2="",PilihNegeri,INDIRECT(SUBSTITUTE(J2," ","_")))</formula1>
     </dataValidation>
   </dataValidations>
 </worksheet>
@@ -438,18 +517,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="3" width="88" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="108" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Import akaun Penternak / Pembekal — Sistem Jejak GPL</t>
+          <t xml:space="preserve">Import akaun syarikat — Sistem Jejak GPL</t>
         </is>
       </c>
     </row>
@@ -466,89 +545,69 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lajur Peranan, Negeri dan Daerah ada senarai pilihan pada setiap baris. Klik anak panah di dalam sel.</t>
+          <t xml:space="preserve">Jenis dalam rantaian sama dengan Profil → Jenis dalam rantaian. Jejak pecahan guna jenis syarikat yang memegang lot itu.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilih Negeri dahulu. Senarai Daerah pada baris itu berubah mengikut negeri. Jika negeri ditukar, pilih semula daerah.</t>
+          <t xml:space="preserve">Jenis dalam rantaian, Negeri dan Daerah ada senarai pilihan pada setiap baris. Klik anak panah di dalam sel.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Perlis, Kuala Lumpur, Labuan dan Putrajaya hanya mempunyai satu pilihan daerah.</t>
+          <t xml:space="preserve">Pilih Negeri dahulu. Senarai Daerah pada baris itu berubah mengikut negeri. Jika negeri ditukar, pilih semula daerah.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t xml:space="preserve">Perlis, Kuala Lumpur, Labuan dan Putrajaya hanya mempunyai satu pilihan daerah.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consumer bukan jenis akaun. Jejak menambah Consumer sendiri bila lot dijual tanpa log masuk syarikat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t xml:space="preserve">Padam baris contoh sebelum guna data sebenar. Jangan hantar fail ini melalui emel kerana ia mengandungi kata laluan.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8"/>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Lajur</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Wajib</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Peraturan</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nama Pengguna</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nama orang yang log masuk.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No. Kad Pengenalan</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ya</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12 digit tanpa sengkang. Lajur ini disimpan sebagai teks.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emel Log Masuk</t>
+          <t xml:space="preserve">Nama Pengguna</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -558,14 +617,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emel unik untuk log masuk. Peranan dalaman akaun ialah Usahawan.</t>
+          <t xml:space="preserve">Nama orang yang log masuk.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kata Laluan</t>
+          <t xml:space="preserve">No. Kad Pengenalan</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -575,14 +634,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Minimum 8 aksara. Minta pengguna tukar selepas log masuk pertama.</t>
+          <t xml:space="preserve">12 digit tanpa sengkang. Lajur ini disimpan sebagai teks.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peranan</t>
+          <t xml:space="preserve">Emel Log Masuk</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -592,14 +651,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dropdown: Pembekal atau Penternak.</t>
+          <t xml:space="preserve">Emel unik untuk log masuk. Peranan dalaman akaun ialah Usahawan.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">No. Pendaftaran</t>
+          <t xml:space="preserve">Kata Laluan</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -609,14 +668,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unik. Nombor akaun luaran dijana sebagai FAMA-&lt;no. pendaftaran&gt;.</t>
+          <t xml:space="preserve">Minimum 8 aksara. Minta pengguna tukar selepas log masuk pertama.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nama Syarikat / Ladang</t>
+          <t xml:space="preserve">Jenis dalam rantaian</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -626,82 +685,82 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nama yang dipaparkan pada syarikat.</t>
+          <t xml:space="preserve">Dropdown: Pengeluar, Pemborong, Peruncit, atau Lain-lain.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alamat</t>
+          <t xml:space="preserve">Nama lapisan</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ya</t>
+          <t xml:space="preserve">Jika Lain-lain</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alamat premis atau ladang.</t>
+          <t xml:space="preserve">Wajib bila jenis ialah Lain-lain. Contoh: Penternak atau Pengumpul. Teks ini yang keluar pada jejak.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Negeri</t>
+          <t xml:space="preserve">No. Pendaftaran</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tidak</t>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dropdown negeri dan wilayah persekutuan.</t>
+          <t xml:space="preserve">Unik. Nombor akaun luaran dijana sebagai FAMA-&lt;no. pendaftaran&gt;.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Daerah</t>
+          <t xml:space="preserve">Nama Syarikat / Ladang</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tidak</t>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dropdown mengikut negeri pada baris yang sama.</t>
+          <t xml:space="preserve">Nama yang dipaparkan pada syarikat.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Poskod</t>
+          <t xml:space="preserve">Alamat</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tidak</t>
+          <t xml:space="preserve">Ya</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Disimpan sebagai teks supaya sifar di hadapan kekal.</t>
+          <t xml:space="preserve">Alamat premis atau ladang.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">No. Telefon</t>
+          <t xml:space="preserve">Negeri</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -711,14 +770,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nombor telefon syarikat.</t>
+          <t xml:space="preserve">Dropdown negeri dan wilayah persekutuan.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emel Syarikat</t>
+          <t xml:space="preserve">Daerah</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -728,14 +787,14 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jika kosong, emel log masuk digunakan untuk syarikat.</t>
+          <t xml:space="preserve">Dropdown mengikut negeri pada baris yang sama.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laman Web</t>
+          <t xml:space="preserve">Poskod</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -745,56 +804,173 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilihan. Contoh: https://ladang.example</t>
+          <t xml:space="preserve">Disimpan sebagai teks supaya sifar di hadapan kekal.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24"/>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Peranan dalam fail</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lapisan syarikat dalam sistem</t>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No. Telefon</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tidak</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nombor telefon syarikat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emel Syarikat</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tidak</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jika kosong, emel log masuk digunakan untuk syarikat.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pembekal</t>
+          <t xml:space="preserve">Laman Web</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPPLIER — label paparan: Pembekal</t>
+          <t xml:space="preserve">Tidak</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilihan. Contoh: https://ladang.example</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Penternak</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OTHER — label paparan: Penternak</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28"/>
+      <c r="A27"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jenis dalam fail</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kod sistem</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paparan pada jejak</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contoh baris ada pada helaian Contoh. Kedua-dua baris contoh juga ada dropdown.</t>
+          <t xml:space="preserve">Pengeluar</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SUPPLIER</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pengeluar</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pemborong</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXPORTER</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pemborong</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peruncit</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RETAILER</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peruncit</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lain-lain</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OTHER</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nama lapisan, contoh Penternak</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consumer</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bukan akaun. Ditambah bila lot dijual tanpa syarikat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contoh pada helaian Contoh: Pengeluar, Pemborong, dan Peruncit. Tiada baris Consumer.</t>
         </is>
       </c>
     </row>
@@ -807,31 +983,31 @@
   <dimension ref="A1:S46"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="18" customWidth="1"/>
-    <col min="13" max="13" width="18" customWidth="1"/>
-    <col min="14" max="14" width="18" customWidth="1"/>
-    <col min="15" max="15" width="18" customWidth="1"/>
-    <col min="16" max="16" width="18" customWidth="1"/>
-    <col min="17" max="17" width="18" customWidth="1"/>
-    <col min="18" max="18" width="18" customWidth="1"/>
-    <col min="19" max="19" width="18" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="14" max="14" width="22" customWidth="1"/>
+    <col min="15" max="15" width="22" customWidth="1"/>
+    <col min="16" max="16" width="22" customWidth="1"/>
+    <col min="17" max="17" width="22" customWidth="1"/>
+    <col min="18" max="18" width="22" customWidth="1"/>
+    <col min="19" max="19" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peranan</t>
+          <t xml:space="preserve">Jenis</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -924,7 +1100,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pembekal</t>
+          <t xml:space="preserve">Pengeluar</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1021,7 +1197,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Penternak</t>
+          <t xml:space="preserve">Pemborong</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1096,7 +1272,11 @@
       <c r="S3"/>
     </row>
     <row r="4">
-      <c r="A4"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peruncit</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
           <t xml:space="preserve">Kelantan</t>
@@ -1169,7 +1349,11 @@
       <c r="S4"/>
     </row>
     <row r="5">
-      <c r="A5"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lain-lain</t>
+        </is>
+      </c>
       <c r="B5" t="inlineStr">
         <is>
           <t xml:space="preserve">Melaka</t>

</xml_diff>